<commit_message>
univariate analysis part 1
</commit_message>
<xml_diff>
--- a/Are Prices Justified - IPL 2026/_dataset/IPL_2026_Combined_Data.xlsx
+++ b/Are Prices Justified - IPL 2026/_dataset/IPL_2026_Combined_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rano's PC\Machine\InsightForge\InsightForge\Are Prices Justified - IPL 2026\_dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60176F27-0518-4398-B4C1-9301C5C33087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000351AC-2844-4174-AB2C-9C9473208A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1761" uniqueCount="512">
   <si>
     <t>POS</t>
   </si>
@@ -1558,6 +1558,9 @@
   </si>
   <si>
     <t xml:space="preserve">Xavier Bartlett  </t>
+  </si>
+  <si>
+    <t>Rajasthan Royals</t>
   </si>
 </sst>
 </file>
@@ -14453,7 +14456,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H174"/>
+  <dimension ref="A1:H179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
@@ -18991,6 +18994,121 @@
         <v>328</v>
       </c>
     </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>15</v>
+      </c>
+      <c r="B175">
+        <v>2025</v>
+      </c>
+      <c r="C175" s="2">
+        <v>3000000</v>
+      </c>
+      <c r="D175" s="2">
+        <v>11000000</v>
+      </c>
+      <c r="E175" t="s">
+        <v>408</v>
+      </c>
+      <c r="F175" t="s">
+        <v>511</v>
+      </c>
+      <c r="G175" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>31</v>
+      </c>
+      <c r="B176">
+        <v>2025</v>
+      </c>
+      <c r="C176" s="2">
+        <v>20000000</v>
+      </c>
+      <c r="D176" s="2">
+        <v>210000000</v>
+      </c>
+      <c r="E176" t="s">
+        <v>408</v>
+      </c>
+      <c r="F176" t="s">
+        <v>411</v>
+      </c>
+      <c r="G176" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>131</v>
+      </c>
+      <c r="B177">
+        <v>2025</v>
+      </c>
+      <c r="C177" s="2">
+        <v>20000000</v>
+      </c>
+      <c r="D177" s="2">
+        <v>163000000</v>
+      </c>
+      <c r="E177" t="s">
+        <v>408</v>
+      </c>
+      <c r="F177" t="s">
+        <v>440</v>
+      </c>
+      <c r="G177" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>141</v>
+      </c>
+      <c r="B178">
+        <v>2025</v>
+      </c>
+      <c r="C178" s="2">
+        <v>20000000</v>
+      </c>
+      <c r="D178" s="2">
+        <v>180000000</v>
+      </c>
+      <c r="E178" t="s">
+        <v>408</v>
+      </c>
+      <c r="F178" t="s">
+        <v>511</v>
+      </c>
+      <c r="G178" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>220</v>
+      </c>
+      <c r="B179">
+        <v>2025</v>
+      </c>
+      <c r="C179" s="2">
+        <v>20000000</v>
+      </c>
+      <c r="D179" s="2">
+        <v>120000000</v>
+      </c>
+      <c r="E179" t="s">
+        <v>408</v>
+      </c>
+      <c r="F179" t="s">
+        <v>418</v>
+      </c>
+      <c r="G179" t="s">
+        <v>415</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="G1:G174" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>